<commit_message>
chore (jdt) : update
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\github\ReadME-MAUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42EB78D9-6205-4419-ADD6-49556356BB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08806EA4-E3DA-4D5B-8DAA-A37991CF84A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="31995" yWindow="0" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -149,6 +149,12 @@
   </si>
   <si>
     <t>Création du projet, et versionning du projet</t>
+  </si>
+  <si>
+    <t>Ajout du grid (place holders) pour les livres sur la page d'accueil</t>
+  </si>
+  <si>
+    <t>Renseignement sur le fonctionnement des fichiers .epub</t>
   </si>
 </sst>
 </file>
@@ -1156,10 +1162,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>20</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>115</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2011,10 +2017,10 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.14814814814814814</c:v>
+                  <c:v>0.16666666666666666</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.85185185185185186</c:v>
+                  <c:v>0.83333333333333337</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4255,7 +4261,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>2 heures 15 minutes</v>
+        <v>4 heures 0 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4270,15 +4276,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>135</v>
+        <v>240</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4420,15 +4426,25 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="63" t="str">
+      <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v/>
-      </c>
-      <c r="B11" s="34"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="23"/>
+        <v>13</v>
+      </c>
+      <c r="B11" s="34">
+        <v>46107</v>
+      </c>
+      <c r="C11" s="35">
+        <v>1</v>
+      </c>
+      <c r="D11" s="36">
+        <v>25</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>36</v>
+      </c>
       <c r="G11" s="40"/>
       <c r="M11" t="s">
         <v>19</v>
@@ -4441,15 +4457,23 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="62" t="str">
+      <c r="A12" s="62">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v/>
-      </c>
-      <c r="B12" s="30"/>
+        <v>13</v>
+      </c>
+      <c r="B12" s="30">
+        <v>46107</v>
+      </c>
       <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="23"/>
+      <c r="D12" s="32">
+        <v>20</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
         <v>20</v>
@@ -10869,11 +10893,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10881,11 +10905,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 20 min</v>
+        <v>0 h 40 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.14814814814814814</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10902,15 +10926,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>115</v>
+        <v>200</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10918,11 +10942,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>1 h 55 min</v>
+        <v>3 h 20 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.85185185185185186</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11048,26 +11072,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>135</v>
+        <v>240</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>31</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>2 h 15 min</v>
+        <v>4 h 00 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>2.5000000000000001E-2</v>
+        <v>4.4444444444444446E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>31</v>
@@ -11106,15 +11130,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11303,6 +11318,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -11315,14 +11339,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11341,6 +11357,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>

</xml_diff>